<commit_message>
paper run 2026-09-07 11:56
</commit_message>
<xml_diff>
--- a/reports/2026-09-07.xlsx
+++ b/reports/2026-09-07.xlsx
@@ -651,13 +651,13 @@
         </is>
       </c>
       <c r="B16" t="n">
+        <v>3</v>
+      </c>
+      <c r="C16" t="n">
         <v>2</v>
       </c>
-      <c r="C16" t="n">
-        <v>1</v>
-      </c>
       <c r="D16" t="n">
-        <v>-9.98</v>
+        <v>25.62</v>
       </c>
       <c r="E16" t="n">
         <v>0</v>
@@ -715,13 +715,13 @@
         </is>
       </c>
       <c r="B20" t="n">
+        <v>3</v>
+      </c>
+      <c r="C20" t="n">
         <v>2</v>
       </c>
-      <c r="C20" t="n">
-        <v>1</v>
-      </c>
       <c r="D20" t="n">
-        <v>-7.02</v>
+        <v>28.58</v>
       </c>
       <c r="E20" t="n">
         <v>0</v>
@@ -741,13 +741,13 @@
         </is>
       </c>
       <c r="B22" t="n">
+        <v>4</v>
+      </c>
+      <c r="C22" t="n">
         <v>3</v>
       </c>
-      <c r="C22" t="n">
-        <v>2</v>
-      </c>
       <c r="D22" t="n">
-        <v>31.55</v>
+        <v>67.15000000000001</v>
       </c>
       <c r="E22" t="n">
         <v>0</v>
@@ -786,13 +786,13 @@
         </is>
       </c>
       <c r="B25" t="n">
+        <v>5</v>
+      </c>
+      <c r="C25" t="n">
         <v>4</v>
       </c>
-      <c r="C25" t="n">
-        <v>3</v>
-      </c>
       <c r="D25" t="n">
-        <v>60.14</v>
+        <v>95.73999999999999</v>
       </c>
       <c r="E25" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
paper run 2026-09-07 23:53
</commit_message>
<xml_diff>
--- a/reports/2026-09-07.xlsx
+++ b/reports/2026-09-07.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -472,6 +472,49 @@
         <is>
           <t>P&amp;L $</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-09-07T22:43:57.093575+00:00</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="F2" t="n">
+        <v>26.68</v>
+      </c>
+      <c r="G2" t="n">
+        <v>51.3</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.00111</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K2" t="n">
+        <v>24.62</v>
       </c>
     </row>
   </sheetData>
@@ -485,7 +528,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -507,7 +550,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -517,7 +560,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -536,6 +579,9 @@
           <t>winrate</t>
         </is>
       </c>
+      <c r="B5" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -544,7 +590,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0</v>
+        <v>24.62</v>
       </c>
     </row>
     <row r="7">
@@ -554,7 +600,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0</v>
+        <v>24.62</v>
       </c>
     </row>
     <row r="8">
@@ -573,6 +619,9 @@
           <t>pf</t>
         </is>
       </c>
+      <c r="B9" t="n">
+        <v>99</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -581,7 +630,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>771.3600000000001</v>
+        <v>795.9800000000001</v>
       </c>
     </row>
     <row r="12">
@@ -632,13 +681,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C15" t="n">
         <v>2</v>
       </c>
       <c r="D15" t="n">
-        <v>70.12</v>
+        <v>31.55</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
@@ -651,16 +700,16 @@
         </is>
       </c>
       <c r="B16" t="n">
+        <v>4</v>
+      </c>
+      <c r="C16" t="n">
         <v>3</v>
       </c>
-      <c r="C16" t="n">
-        <v>2</v>
-      </c>
       <c r="D16" t="n">
-        <v>25.62</v>
+        <v>61.22</v>
       </c>
       <c r="E16" t="n">
-        <v>0</v>
+        <v>24.62</v>
       </c>
     </row>
     <row r="17">
@@ -696,16 +745,16 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D19" t="n">
-        <v>28.59</v>
+        <v>64.19</v>
       </c>
       <c r="E19" t="n">
-        <v>0</v>
+        <v>24.62</v>
       </c>
     </row>
     <row r="20">
@@ -715,13 +764,13 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C20" t="n">
         <v>2</v>
       </c>
       <c r="D20" t="n">
-        <v>28.58</v>
+        <v>-9.99</v>
       </c>
       <c r="E20" t="n">
         <v>0</v>
@@ -741,16 +790,16 @@
         </is>
       </c>
       <c r="B22" t="n">
+        <v>6</v>
+      </c>
+      <c r="C22" t="n">
         <v>4</v>
       </c>
-      <c r="C22" t="n">
-        <v>3</v>
-      </c>
       <c r="D22" t="n">
-        <v>67.15000000000001</v>
+        <v>64.18000000000001</v>
       </c>
       <c r="E22" t="n">
-        <v>0</v>
+        <v>24.62</v>
       </c>
     </row>
     <row r="23">
@@ -786,42 +835,61 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C25" t="n">
         <v>4</v>
       </c>
       <c r="D25" t="n">
-        <v>95.73999999999999</v>
+        <v>57.17</v>
       </c>
       <c r="E25" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>1</v>
+      </c>
+      <c r="C26" t="n">
+        <v>1</v>
+      </c>
+      <c r="D26" t="n">
+        <v>35.6</v>
+      </c>
+      <c r="E26" t="n">
+        <v>24.62</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
         <is>
           <t>REALIZED (реальные сделки)</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
+    <row r="30">
+      <c r="A30" t="inlineStr">
         <is>
           <t>По активам</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B30" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D30" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
@@ -830,64 +898,74 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>По окнам</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>1</v>
+      </c>
+      <c r="C31" t="n">
+        <v>1</v>
+      </c>
+      <c r="D31" t="n">
+        <v>24.62</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
+          <t>По окнам</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>5m</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>1</v>
+      </c>
+      <c r="C34" t="n">
+        <v>1</v>
+      </c>
+      <c r="D34" t="n">
+        <v>24.62</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
           <t>По часам</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B36" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C36" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>По цене входа</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
+      <c r="D36" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
@@ -896,45 +974,131 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>По силе движения</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>1</v>
+      </c>
+      <c r="C37" t="n">
+        <v>1</v>
+      </c>
+      <c r="D37" t="n">
+        <v>24.62</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
+          <t>По цене входа</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>0.50–0.55</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>1</v>
+      </c>
+      <c r="C40" t="n">
+        <v>1</v>
+      </c>
+      <c r="D40" t="n">
+        <v>24.62</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>По силе движения</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>0.10–0.12%</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>1</v>
+      </c>
+      <c r="C43" t="n">
+        <v>1</v>
+      </c>
+      <c r="D43" t="n">
+        <v>24.62</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
           <t>По направлению</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="B45" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C45" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="D45" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>1</v>
+      </c>
+      <c r="C46" t="n">
+        <v>1</v>
+      </c>
+      <c r="D46" t="n">
+        <v>24.62</v>
       </c>
     </row>
   </sheetData>

</xml_diff>